<commit_message>
[agenthub/cleanup-tools-gemini] 트랙 #84-2 — 운영 mutation cleanup + Tools/Dockerfile/Agent 코드 보강 + deploy + 재검증
상세:
- 운영 cleanup: Tools 8 + Agents 4 + ApiKey 1 DELETE (test-track84-* 잔존, ApiKey3 docutil-runtime-key 보존)
- ToolExecutionService → ToolNotFoundException/ToolVersionNotActiveException 도메인 예외 분리
- ToolsController.ExecuteTool: 도메인 예외 catch 404/400 한국어 매핑
- AgentsController.CreateAgent: ServiceId FK 사전 검증 + DbUpdateException 이중 안전망
- Dockerfile runtime: python3 + python3-pip 추가 (ScriptToolExecutor 대비)
- AiProxyService.Gemini: 점검 후 변경 보류 (historical, 운영 매치 0, 명확한 결함 미발견)
- 운영 IIS 재배포 + Playwright 87 routes PASS 65 / FAIL 0 / SKIP 22 (console errors 0, network 5xx 0)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TEST_CHECKLIST_FULL.xlsx
+++ b/docs/TEST_CHECKLIST_FULL.xlsx
@@ -8382,10 +8382,14 @@
           <t>DOM mounted=True | duration=1801ms | final=http://192.168.10.39:64005/agents/builder</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:36</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -8504,10 +8508,14 @@
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:36</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -8559,10 +8567,14 @@
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:36</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -8898,10 +8910,14 @@
           <t>DOM mounted=True | duration=2727ms | final=http://192.168.10.39:64005/agents/chat</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:31</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -9020,10 +9036,14 @@
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:31</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -9075,10 +9095,14 @@
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:31</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -10328,10 +10352,14 @@
           <t>DOM mounted=True | duration=1813ms | final=http://192.168.10.39:64005/agents/multi-chat</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:34</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -10450,10 +10478,14 @@
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:34</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -10505,10 +10537,14 @@
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:34</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -12097,10 +12133,14 @@
           <t>DOM mounted=True | duration=1814ms | final=http://192.168.10.39:64005/agents</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:29</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -12215,10 +12255,14 @@
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:29</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -12270,10 +12314,14 @@
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>[트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 15:32:29</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -36333,12 +36381,12 @@
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:20</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -36459,12 +36507,12 @@
       <c r="J4" s="8" t="inlineStr"/>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:20</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -36518,12 +36566,12 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:20</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
@@ -38933,12 +38981,12 @@
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:23</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -39059,12 +39107,12 @@
       <c r="J4" s="8" t="inlineStr"/>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:23</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
@@ -39118,12 +39166,12 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건</t>
+          <t>[트랙 #84-1] 직전 5xx/401 결함 fix 후 재검증 통과 — console/network 결함 0건 | [트랙 #84-2] 운영 mutation cleanup (Tools 8 + Agents 4 + ApiKey 1 DELETE, ApiKey3 docutil-runtime-key 보존) + ToolExecution 도메인 예외 분리 + AgentsController.CreateAgent ServiceId FK 사전 검증 + Dockerfile python3 추가 — 재배포 후 87 routes PASS 65 / FAIL 0 / SKIP 22, console errors 0, network 5xx 0</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-12 17:02:23</t>
+          <t>2026-05-12 (트랙 #84-2 재검증)</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr"/>

</xml_diff>